<commit_message>
feat: login peserta didik dengan NISN (username & kata sandi awal)
- Auth.js: kolom login menerima email ATAU NISN; NISN di-resolve lewat
  tabel students (bukan tebakan email), role lain tetap pakai email
- Pembuatan siswa (satuan & impor Excel): email/password dihapus dari
  form; akun dibuat otomatis (email internal <nisn>@siswa.internal,
  kata sandi awal = NISN); NISN wajib 5-30 digit & unik (migrasi 0002)
- PATCH /students/:id/reset-password: reset sandi siswa lama ke NISN,
  tombol per baris di daftar siswa admin
- Impor Excel: NIS/NISN dinormalisasi ke string (Excel membaca angka),
  template docs/templates/template-import-siswa.xlsx dibuat ulang
- shared: nisnToEmail/NISN_REGEX di packages/shared/src/students.ts
- Dokumentasi: tutorial & bulk-import-export diperbarui + catatan
  keamanan (password=NISN hanya sandi awal, ganti sandi menyusul Fase 9)
</commit_message>
<xml_diff>
--- a/docs/templates/template-import-siswa.xlsx
+++ b/docs/templates/template-import-siswa.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +49,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,158 +418,126 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="37" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>password</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>nis</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>nisn</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>fullName</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>className</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>gradeLevel</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>gender</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>birthDate</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>budi.santoso@siswa.sekolah.sch.id</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>sandiawal123</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>0123456789</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026001</t>
+          <t>Ahmad Fauzi</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0091234567</t>
+          <t>VII A</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Budi Santoso</t>
+          <t>VII</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>VII A</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>VII</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2013-05-14</t>
+          <t>2013-04-12</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>siti.aminah@siswa.sekolah.sch.id</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>sandiawal123</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>0123456790</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026002</t>
+          <t>Siti Rahma</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0091234568</t>
+          <t>VII B</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Siti Aminah</t>
+          <t>VII</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>VII A</t>
+          <t>P</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>VII</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2013-08-02</t>
+          <t>2013-09-30</t>
         </is>
       </c>
     </row>

</xml_diff>